<commit_message>
fix(maker): exclude PPN dari total_penawaran + INFO status di math check
Masalah: dokumen penawaran dengan PPN 11% di baris TOTAL memicu false
positive 'Inkonsistensi Matematis' karena total_penawaran (83.25jt) !=
sum(items) (75jt). Selisih persis PPN.

Fix:
- Tambah konstanta _MAKER_PROMPT_PENAWARAN, override Prompt Template-J026A
  di mode penawaran. Prompt tegas: items HANYA barang/jasa (bukan
  Subtotal/PPN/TOTAL), total_penawaran = sum(items.total_price_vendor).
- _apply_math_check: range 9-13% selisih -> status INFO (kemungkinan PPN),
  bukan CRITICAL.
- Frontend MathCheckBanner: handle status INFO (border electric), plus
  fix warna warning/critical -> amber + sev-critical.
- Sample BON v2 Excel untuk demo PDF-flow.

Verified: Excel penawaran PPN 11% -> total_penawaran 75jt, math OK.
</commit_message>
<xml_diff>
--- a/sample-docs/13-Pengajuan-Rabu-30-Sept-2026-bon-v2.xlsx
+++ b/sample-docs/13-Pengajuan-Rabu-30-Sept-2026-bon-v2.xlsx
@@ -425,16 +425,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -611,6 +611,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -618,16 +619,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -754,6 +755,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -761,16 +763,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -878,5 +880,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>